<commit_message>
fix(test-fixtures): use null-id row to force float64, not fractional values
Revert phone numbers to whole integers. Add one empty-id row to each fixture
(users and survey) to reproduce the real export's float64 dtype inference
via nullable numeric type, not via fractional values.

The null-id row forces pandas to read Address/Respondent as float64 because
the NA value in a numeric column triggers float inference. This preserves
byte-identical phone number values across fixtures (fixing user 5 mismatch
between fixtures) and allows Task 4's load.digits() to work correctly without
encoding the bug it's designed to catch.

Update test counts: 7 rows for users (6 + 1 null), 5 rows for survey (4 + 1 null).
Null-id rows are not counted in v1/v2 cohort assertions.
</commit_message>
<xml_diff>
--- a/tests/fixtures/survey_v2.xlsx
+++ b/tests/fixtures/survey_v2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,7 +615,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>571110000005.5</v>
+        <v>571110000005</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -636,6 +636,11 @@
         <is>
           <t>Recomendación de ONG</t>
         </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="M8" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>